<commit_message>
feat maintain non equipment create
</commit_message>
<xml_diff>
--- a/docs/SLMS2026_import_matrix_dot1.xlsx
+++ b/docs/SLMS2026_import_matrix_dot1.xlsx
@@ -401,14 +401,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <cols>
-    <col min="1" max="1" width="51.83203125" customWidth="1"/>
+    <col min="1" max="1" width="56.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Hướng dẫn — Ma trận đủ 10 TH onboarding (đợt 1)</v>
+        <v>Hướng dẫn — Ma trận onboarding + căn full NT (đợt 1)</v>
       </c>
     </row>
     <row r="2">
@@ -418,12 +418,12 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>File này cover đủ 10 trường hợp hợp lệ theo logic import SLMS2026.</v>
+        <v>File cover #1–#10 ma trận hợp lệ + #11–#14 nội thất đầy đủ.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Sheet "0. Ma_Tran_Onboarding": tra cứu STT #1–#10.</v>
+        <v>Sheet "0. Ma_Tran_Onboarding": tra cứu STT.</v>
       </c>
     </row>
     <row r="5">
@@ -438,24 +438,29 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>#1–#2 NORENO: sau đợt 1 tự gửi Host — KHÔNG import file đợt 2.</v>
+        <v>#1–#2, #11 NORENO: sau đợt 1 tự gửi Host — KHÔNG import file đợt 2.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>#3–#10 RENO: sau đợt 1 ở UNDER_RENOVATION — cần file đợt 2.</v>
+        <v>#3–#10, #12–#14 RENO: sau đợt 1 ở UNDER_RENOVATION — cần file đợt 2.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>#13–#14 THEO_PHONG: mỗi phòng có 1 Quạt + 1 Giường (sheet TB mua đợt 2).</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A9"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I20"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -788,28 +793,149 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="str">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>HD-MTX-11-NORENO-FULL</v>
+      </c>
+      <c r="C12" t="str">
+        <v>NORENO</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Có</v>
+      </c>
+      <c r="E12" t="str">
+        <v>—</v>
+      </c>
+      <c r="F12" t="str">
+        <v>—</v>
+      </c>
+      <c r="G12" t="str">
+        <v>—</v>
+      </c>
+      <c r="H12" t="str">
+        <v>Không</v>
+      </c>
+      <c r="I12" t="str">
+        <v>#11 NORENO | Nguyên căn full NT bàn giao | Đợt 2: —</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>HD-MTX-12-RENO-WH-FULL</v>
+      </c>
+      <c r="C13" t="str">
+        <v>RENO</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Có</v>
+      </c>
+      <c r="E13" t="str">
+        <v>NGUYEN_CAN</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Có (≥1 dòng)</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Có</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Có</v>
+      </c>
+      <c r="I13" t="str">
+        <v>#12 RENO | NGUYEN_CAN full NT | TB bàn giao + cải tạo + TB mua khu vực chung</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>HD-MTX-13-RENO-RM-FULL</v>
+      </c>
+      <c r="C14" t="str">
+        <v>RENO</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Có</v>
+      </c>
+      <c r="E14" t="str">
+        <v>THEO_PHONG (4)</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Có (≥1 dòng)</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Có</v>
+      </c>
+      <c r="H14" t="str">
+        <v>Có</v>
+      </c>
+      <c r="I14" t="str">
+        <v>#13 RENO | THEO_PHONG (4) full NT | mỗi phòng 1 Quạt + 1 Giường (+ ĐH, nóng lạnh)</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>HD-MTX-14-RENO-RM-BEDFAN</v>
+      </c>
+      <c r="C15" t="str">
+        <v>RENO</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Không</v>
+      </c>
+      <c r="E15" t="str">
+        <v>THEO_PHONG (5)</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Có (≥1 dòng)</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Có</v>
+      </c>
+      <c r="H15" t="str">
+        <v>Có</v>
+      </c>
+      <c r="I15" t="str">
+        <v>#14 RENO | THEO_PHONG (5) | mỗi phòng đúng 1 Quạt + 1 Giường</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
         <v/>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Tổng: 10 trường hợp onboarding hợp lệ (2 NORENO + 8 RENO).</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Tổng: 14 HĐ onboarding (#1–#10 ma trận + #11–#14 nội thất đầy đủ).</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
         <v>NORENO: import đợt 1 xong → tự gửi Host. RENO: cần import đợt 2.</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="str">
+    <row r="19">
+      <c r="A19" t="str">
         <v>RENO bắt buộc ≥1 hạng mục cải tạo ở sheet 3 trước khi gửi Host.</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>#11–#14: demo full NT — nguyên căn / theo phòng (mỗi phòng ≥ 1 Quạt + 1 Giường).</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I20"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -932,7 +1058,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:O15"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -1468,16 +1594,204 @@
         <v>Ma trận #10 — RENO THEO_PHONG 3 phòng đầy đủ.</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>HD-MTX-11-NORENO-FULL</v>
+      </c>
+      <c r="B12" t="str">
+        <v>MTX#11 NORENO full NT</v>
+      </c>
+      <c r="C12" t="str">
+        <v>11 Ma Trận Tân Bình</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Tân Bình</v>
+      </c>
+      <c r="E12" t="str">
+        <v>TP. Hồ Chí Minh</v>
+      </c>
+      <c r="F12">
+        <v>95</v>
+      </c>
+      <c r="G12">
+        <v>11.5</v>
+      </c>
+      <c r="H12">
+        <v>8.3</v>
+      </c>
+      <c r="I12">
+        <v>2</v>
+      </c>
+      <c r="J12">
+        <v>4</v>
+      </c>
+      <c r="K12" t="str">
+        <v>Lý Văn L</v>
+      </c>
+      <c r="L12">
+        <v>250000000</v>
+      </c>
+      <c r="M12" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="N12" t="str">
+        <v>2028-07-31</v>
+      </c>
+      <c r="O12" t="str">
+        <v>Ma trận #11 — NORENO nguyên căn, nội thất đầy đủ từ chủ (bàn giao).</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>HD-MTX-12-RENO-WH-FULL</v>
+      </c>
+      <c r="B13" t="str">
+        <v>MTX#12 NGUYEN_CAN full NT</v>
+      </c>
+      <c r="C13" t="str">
+        <v>12 Ma Trận Tân Bình</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Tân Bình</v>
+      </c>
+      <c r="E13" t="str">
+        <v>TP. Hồ Chí Minh</v>
+      </c>
+      <c r="F13">
+        <v>110</v>
+      </c>
+      <c r="G13">
+        <v>12.4</v>
+      </c>
+      <c r="H13">
+        <v>8.9</v>
+      </c>
+      <c r="I13">
+        <v>2</v>
+      </c>
+      <c r="J13">
+        <v>4</v>
+      </c>
+      <c r="K13" t="str">
+        <v>Mai Thị M</v>
+      </c>
+      <c r="L13">
+        <v>280000000</v>
+      </c>
+      <c r="M13" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="N13" t="str">
+        <v>2028-07-31</v>
+      </c>
+      <c r="O13" t="str">
+        <v>Ma trận #12 — RENO NGUYEN_CAN nội thất đầy đủ: TB chủ + cải tạo + mua TB khu vực chung.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>HD-MTX-13-RENO-RM-FULL</v>
+      </c>
+      <c r="B14" t="str">
+        <v>MTX#13 THEO_PHONG full NT</v>
+      </c>
+      <c r="C14" t="str">
+        <v>13 Ma Trận Thủ Đức</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Thủ Đức</v>
+      </c>
+      <c r="E14" t="str">
+        <v>TP. Hồ Chí Minh</v>
+      </c>
+      <c r="F14">
+        <v>120</v>
+      </c>
+      <c r="G14">
+        <v>13</v>
+      </c>
+      <c r="H14">
+        <v>9.2</v>
+      </c>
+      <c r="I14">
+        <v>3</v>
+      </c>
+      <c r="J14">
+        <v>6</v>
+      </c>
+      <c r="K14" t="str">
+        <v>Phan Văn N</v>
+      </c>
+      <c r="L14">
+        <v>320000000</v>
+      </c>
+      <c r="M14" t="str">
+        <v>2026-09-01</v>
+      </c>
+      <c r="N14" t="str">
+        <v>2028-08-31</v>
+      </c>
+      <c r="O14" t="str">
+        <v>Ma trận #13 — RENO THEO_PHONG 4 phòng, mỗi phòng mua 1 Quạt + 1 Giường (+ ĐH/nóng lạnh).</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>HD-MTX-14-RENO-RM-BEDFAN</v>
+      </c>
+      <c r="B15" t="str">
+        <v>MTX#14 THEO_PHONG giường+quạt</v>
+      </c>
+      <c r="C15" t="str">
+        <v>14 Ma Trận Thủ Đức</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Thủ Đức</v>
+      </c>
+      <c r="E15" t="str">
+        <v>TP. Hồ Chí Minh</v>
+      </c>
+      <c r="F15">
+        <v>90</v>
+      </c>
+      <c r="G15">
+        <v>11.2</v>
+      </c>
+      <c r="H15">
+        <v>8</v>
+      </c>
+      <c r="I15">
+        <v>2</v>
+      </c>
+      <c r="J15">
+        <v>5</v>
+      </c>
+      <c r="K15" t="str">
+        <v>Trịnh Thị O</v>
+      </c>
+      <c r="L15">
+        <v>240000000</v>
+      </c>
+      <c r="M15" t="str">
+        <v>2026-09-01</v>
+      </c>
+      <c r="N15" t="str">
+        <v>2028-08-31</v>
+      </c>
+      <c r="O15" t="str">
+        <v>Ma trận #14 — RENO THEO_PHONG 5 phòng, mỗi phòng đúng 1 Quạt + 1 Giường.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O15"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G25"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -1672,9 +1986,400 @@
         <v/>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>HD-MTX-11-NORENO-FULL</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Điều hòa</v>
+      </c>
+      <c r="C9" t="str">
+        <v>1.5HP Inverter</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Phòng khách</v>
+      </c>
+      <c r="E9" t="str">
+        <v>GOOD</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>HD-MTX-11-NORENO-FULL</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Điều hòa</v>
+      </c>
+      <c r="C10" t="str">
+        <v>1HP</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Phòng ngủ 1</v>
+      </c>
+      <c r="E10" t="str">
+        <v>GOOD</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>HD-MTX-11-NORENO-FULL</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Tủ lạnh</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Inverter 200L</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Bếp</v>
+      </c>
+      <c r="E11" t="str">
+        <v>GOOD</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>HD-MTX-11-NORENO-FULL</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Máy giặt</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Cửa trước 8kg</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Sân sau</v>
+      </c>
+      <c r="E12" t="str">
+        <v>GOOD</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>HD-MTX-11-NORENO-FULL</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Nóng lạnh</v>
+      </c>
+      <c r="C13" t="str">
+        <v>15L</v>
+      </c>
+      <c r="D13" t="str">
+        <v>WC tầng 1</v>
+      </c>
+      <c r="E13" t="str">
+        <v>GOOD</v>
+      </c>
+      <c r="F13">
+        <v>1</v>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>HD-MTX-11-NORENO-FULL</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Giường</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Giường gỗ 1m6</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Phòng ngủ 1</v>
+      </c>
+      <c r="E14" t="str">
+        <v>GOOD</v>
+      </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>HD-MTX-11-NORENO-FULL</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Giường</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Giường gỗ 1m6</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Phòng ngủ 2</v>
+      </c>
+      <c r="E15" t="str">
+        <v>GOOD</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>HD-MTX-11-NORENO-FULL</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Giường</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Giường gỗ 1m2</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Phòng ngủ 3</v>
+      </c>
+      <c r="E16" t="str">
+        <v>GOOD</v>
+      </c>
+      <c r="F16">
+        <v>1</v>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>HD-MTX-11-NORENO-FULL</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Quạt</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Quạt trần</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Phòng khách</v>
+      </c>
+      <c r="E17" t="str">
+        <v>GOOD</v>
+      </c>
+      <c r="F17">
+        <v>1</v>
+      </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>HD-MTX-11-NORENO-FULL</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Quạt</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Quạt đứng</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Phòng ngủ 1</v>
+      </c>
+      <c r="E18" t="str">
+        <v>GOOD</v>
+      </c>
+      <c r="F18">
+        <v>1</v>
+      </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>HD-MTX-11-NORENO-FULL</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Quạt</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Quạt đứng</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Phòng ngủ 2</v>
+      </c>
+      <c r="E19" t="str">
+        <v>GOOD</v>
+      </c>
+      <c r="F19">
+        <v>1</v>
+      </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>HD-MTX-11-NORENO-FULL</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Quạt</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Quạt đứng</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Phòng ngủ 3</v>
+      </c>
+      <c r="E20" t="str">
+        <v>GOOD</v>
+      </c>
+      <c r="F20">
+        <v>1</v>
+      </c>
+      <c r="G20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>HD-MTX-12-RENO-WH-FULL</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Giường</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Giường gỗ cũ</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Phòng ngủ chính</v>
+      </c>
+      <c r="E21" t="str">
+        <v>GOOD</v>
+      </c>
+      <c r="F21">
+        <v>2</v>
+      </c>
+      <c r="G21" t="str">
+        <v>TB chủ giữ lại</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>HD-MTX-12-RENO-WH-FULL</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Quạt</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Quạt trần cũ</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Phòng khách</v>
+      </c>
+      <c r="E22" t="str">
+        <v>GOOD</v>
+      </c>
+      <c r="F22">
+        <v>1</v>
+      </c>
+      <c r="G22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>HD-MTX-12-RENO-WH-FULL</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Tủ lạnh</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Tủ 150L cũ</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Bếp</v>
+      </c>
+      <c r="E23" t="str">
+        <v>DAMAGED</v>
+      </c>
+      <c r="F23">
+        <v>1</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Sắp thay</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>HD-MTX-13-RENO-RM-FULL</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Máy giặt</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Máy cũ chung</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Sân phơi</v>
+      </c>
+      <c r="E24" t="str">
+        <v>GOOD</v>
+      </c>
+      <c r="F24">
+        <v>1</v>
+      </c>
+      <c r="G24" t="str">
+        <v>TB dùng chung</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>HD-MTX-13-RENO-RM-FULL</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Tủ lạnh</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Tủ cũ tầng 1</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Bếp chung</v>
+      </c>
+      <c r="E25" t="str">
+        <v>GOOD</v>
+      </c>
+      <c r="F25">
+        <v>1</v>
+      </c>
+      <c r="G25" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G25"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>